<commit_message>
Add 11 source-reviewed SEU profiles with bounded degree and guidance evidence
</commit_message>
<xml_diff>
--- a/site/exports/seu-humanities-philosophy-science.xlsx
+++ b/site/exports/seu-humanities-philosophy-science.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'导师'!$A$1:$L$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -622,11 +622,65 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>卞绍斌</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>校区未标注</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>人文学院哲学与科学系</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>https://rwxy.seu.edu.cn/2019/0424/c8790a270725/page.htm</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>官网称东南大学人文学院哲学与科学系教授、博士生导师；教授为职称，博导为指导他人的资格，不另造任职或本人师承，起任年月未给。；本批仅保留首个个人页必要片段，教育和本人导师未披露；未读取下一页，不能说完整履历没有教育。；页面显示2019-04-24，所选两部作品原列2024，最后修改时间未知，不用任一日期覆盖另一事实。；两部代表作品仅原专著标签与出版社、年份、版次；完整作者、出版者元数据及全文未核。</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>公开个人页（访问与内容时效见来源记录）</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>seu</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>东南大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K3"/>
+  <autoFilter ref="A1:K4"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1410,7 +1464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1422,7 +1476,7 @@
     <col width="65" customWidth="1" min="7" max="7"/>
     <col width="50.4" customWidth="1" min="8" max="8"/>
     <col width="65" customWidth="1" min="9" max="9"/>
-    <col width="44.8" customWidth="1" min="10" max="10"/>
+    <col width="65" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
@@ -1705,8 +1759,112 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>卞绍斌</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>马克思的社会概念</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>https://rwxy.seu.edu.cn/2019/0424/c8790a270725/page.htm</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>书籍；book</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>https://rwxy.seu.edu.cn/2019/0424/c8790a270725/page.htm</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>官网书目，未核出版者元数据或全文；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>官网代表作品列为专著，完整作者名单及本人具体著编角色未独立核验；商务印书馆，2024年，增订版。不把页面显示2019-04-24当作品年份或最后更新时间。</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>seu</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>东南大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>卞绍斌</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>自律与客观性：寻求社会团结的规范基础</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>https://rwxy.seu.edu.cn/2019/0424/c8790a270725/page.htm</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>书籍；book</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>https://rwxy.seu.edu.cn/2019/0424/c8790a270725/page.htm</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>官网书目，未核出版者元数据或全文；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>官网代表作品列为专著，完整作者名单及本人具体著编角色未独立核验；商务印书馆，2024年。不把页面显示2019-04-24当作品年份或最后更新时间。</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>seu</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>东南大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L5"/>
+  <autoFilter ref="A1:L7"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
@@ -1718,6 +1876,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1729,11 +1891,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18.2" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
     <col width="65" customWidth="1" min="3" max="3"/>
     <col width="65" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -1885,12 +2047,50 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>卞绍斌</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>seu-bianshaobin</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>https://rwxy.seu.edu.cn/2019/0424/c8790a270725/page.htm</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>retained_professional_excerpts_checked</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>seu</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>东南大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G4"/>
+  <autoFilter ref="A1:G5"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>